<commit_message>
feat: semantic model 지속적 개선 중, db별 semantic model 추가, gold sql few shot
</commit_message>
<xml_diff>
--- a/evaluation_history_v4.xlsx
+++ b/evaluation_history_v4.xlsx
@@ -11,6 +11,7 @@
     <sheet name="ipl" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="General" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="bank" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="baseball" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -431,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <sheetData>
     <row r="1">
@@ -1003,6 +1004,66 @@
         <v>1</v>
       </c>
       <c r="R9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-05 23:24:38</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0505_city</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>90</v>
+      </c>
+      <c r="D10" t="n">
+        <v>80</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>9</v>
+      </c>
+      <c r="H10" t="n">
+        <v>10</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1017,7 +1078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EM4"/>
+  <dimension ref="A1:EM5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <sheetData>
     <row r="1">
@@ -3015,6 +3076,102 @@
         <v>0</v>
       </c>
       <c r="EM4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-06 16:33:23</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0506_local_tc_25</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>59.09</v>
+      </c>
+      <c r="D5" t="n">
+        <v>59.09</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>13</v>
+      </c>
+      <c r="H5" t="n">
+        <v>22</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" t="n">
+        <v>1</v>
+      </c>
+      <c r="U5" t="n">
+        <v>1</v>
+      </c>
+      <c r="V5" t="n">
+        <v>1</v>
+      </c>
+      <c r="W5" t="n">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3203,7 +3360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W15"/>
+  <dimension ref="A1:BO29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <sheetData>
     <row r="1">
@@ -3322,6 +3479,226 @@
           <t>local074</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>local007</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>local098</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>local258</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>local253</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>local026</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>local259</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>local309</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>local356</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>local077</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>local009</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>local039</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>local061</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>local063</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>local002</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>local003</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>local015</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>local017</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>local018</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>local029</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>local037</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>local050</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>local097</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>local100</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>local130</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>local131</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>local152</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>local194</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>local201</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>local209</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>local220</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>local244</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>local272</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>local273</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>local277</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>local279</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>local283</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>local286</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>local329</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>local331</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>local335</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>local336</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>local344</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>local358</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>local360</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3823,23 +4200,737 @@
       <c r="H15" t="n">
         <v>1</v>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
       <c r="U15" t="n">
         <v>0</v>
       </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-06 12:15:24</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0506_local_tcc_mini</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="D16" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-06 13:56:58</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0506_local_tcc_mini</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>25</v>
+      </c>
+      <c r="D17" t="n">
+        <v>25</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-06 14:24:46</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0506_local_tcc_mini2</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-06 15:01:26</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0506_local_tcc_mini5</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>5</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-06 15:05:09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0506_local_tcc_mini6</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-06 15:24:56</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0506_local_tcc_mini8</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-06 15:32:30</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0506_local_tcc_mini9</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>25</v>
+      </c>
+      <c r="D22" t="n">
+        <v>25</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>4</v>
+      </c>
+      <c r="M22" t="n">
+        <v>1</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-06 15:37:06</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0506_local077</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-06 15:39:34</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0506_local077_2</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>100</v>
+      </c>
+      <c r="D24" t="n">
+        <v>100</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-06 16:44:43</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0506_local077</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>80</v>
+      </c>
+      <c r="D25" t="n">
+        <v>20</v>
+      </c>
+      <c r="E25" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-06 17:15:20</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0506_test4</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>25</v>
+      </c>
+      <c r="D26" t="n">
+        <v>25</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-06 17:55:53</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0506_test4__</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="D27" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="F27" t="n">
+        <v>4</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-06 20:35:27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0506_local_hardd</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" t="n">
+        <v>42</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-06 20:52:18</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0506_local_mini_</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="D29" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
+      <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr"/>
+      <c r="AG29" t="inlineStr"/>
+      <c r="AH29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI29" t="inlineStr"/>
+      <c r="AJ29" t="inlineStr"/>
+      <c r="AK29" t="inlineStr"/>
+      <c r="AL29" t="inlineStr"/>
+      <c r="AM29" t="inlineStr"/>
+      <c r="AN29" t="inlineStr"/>
+      <c r="AO29" t="inlineStr"/>
+      <c r="AP29" t="inlineStr"/>
+      <c r="AQ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR29" t="inlineStr"/>
+      <c r="AS29" t="inlineStr"/>
+      <c r="AT29" t="inlineStr"/>
+      <c r="AU29" t="inlineStr"/>
+      <c r="AV29" t="inlineStr"/>
+      <c r="AW29" t="inlineStr"/>
+      <c r="AX29" t="inlineStr"/>
+      <c r="AY29" t="inlineStr"/>
+      <c r="AZ29" t="inlineStr"/>
+      <c r="BA29" t="inlineStr"/>
+      <c r="BB29" t="inlineStr"/>
+      <c r="BC29" t="inlineStr"/>
+      <c r="BD29" t="inlineStr"/>
+      <c r="BE29" t="inlineStr"/>
+      <c r="BF29" t="inlineStr"/>
+      <c r="BG29" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH29" t="inlineStr"/>
+      <c r="BI29" t="inlineStr"/>
+      <c r="BJ29" t="inlineStr"/>
+      <c r="BK29" t="inlineStr"/>
+      <c r="BL29" t="inlineStr"/>
+      <c r="BM29" t="inlineStr"/>
+      <c r="BN29" t="inlineStr"/>
+      <c r="BO29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5091,4 +6182,205 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Run Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Final Score (%)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Zero-Retry Score (%)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Avg Retries</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Avg Steps</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>local007</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>local008</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-05 20:51:20</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0505_baseball</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-05 21:03:20</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0505_007</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-05 21:20:04</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0505_007_3</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-05 21:34:07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0505_007_4</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: 마스킹 gold Fewshot
</commit_message>
<xml_diff>
--- a/evaluation_history_v4.xlsx
+++ b/evaluation_history_v4.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <sheetData>
     <row r="1">
@@ -1064,6 +1064,123 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-11 16:08:38</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0511_city</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>90</v>
+      </c>
+      <c r="D11" t="n">
+        <v>60</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" t="n">
+        <v>9</v>
+      </c>
+      <c r="H11" t="n">
+        <v>10</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-25 23:01:01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0525_city2</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>100</v>
+      </c>
+      <c r="D12" t="n">
+        <v>77.78</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" t="n">
+        <v>9</v>
+      </c>
+      <c r="H12" t="n">
+        <v>9</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1078,7 +1195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EM5"/>
+  <dimension ref="A1:EM7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <sheetData>
     <row r="1">
@@ -3172,6 +3289,456 @@
         <v>1</v>
       </c>
       <c r="AE5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:27:32</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0526_local_half</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>57.33</v>
+      </c>
+      <c r="D6" t="n">
+        <v>42.67</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>43</v>
+      </c>
+      <c r="H6" t="n">
+        <v>75</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BZ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CT6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CU6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CW6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CX6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DD6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DE6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DF6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DG6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DH6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DK6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DO6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DP6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DW6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DX6" t="n">
+        <v>1</v>
+      </c>
+      <c r="DY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DZ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="EA6" t="n">
+        <v>1</v>
+      </c>
+      <c r="EB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="EC6" t="n">
+        <v>1</v>
+      </c>
+      <c r="ED6" t="n">
+        <v>0</v>
+      </c>
+      <c r="EE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="EF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="EG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="EH6" t="n">
+        <v>1</v>
+      </c>
+      <c r="EI6" t="n">
+        <v>1</v>
+      </c>
+      <c r="EJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="EK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="EL6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-26 21:48:34</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0526_local_tc2</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>72.73</v>
+      </c>
+      <c r="D7" t="n">
+        <v>54.55</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="G7" t="n">
+        <v>40</v>
+      </c>
+      <c r="H7" t="n">
+        <v>55</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>1</v>
+      </c>
+      <c r="T7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CL7" t="n">
+        <v>1</v>
+      </c>
+      <c r="DS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DV7" t="n">
+        <v>1</v>
+      </c>
+      <c r="EM7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3360,7 +3927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO29"/>
+  <dimension ref="A1:BY37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <sheetData>
     <row r="1">
@@ -3699,6 +4266,56 @@
           <t>local360</t>
         </is>
       </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>local010</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>local060</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>local275</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>local073</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>local210</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>local230</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>local025</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>local096</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr">
+        <is>
+          <t>local311</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>local354</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4866,71 +5483,644 @@
       <c r="H29" t="n">
         <v>3</v>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="inlineStr"/>
-      <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="inlineStr"/>
-      <c r="AB29" t="inlineStr"/>
-      <c r="AC29" t="inlineStr"/>
-      <c r="AD29" t="inlineStr"/>
-      <c r="AE29" t="inlineStr"/>
-      <c r="AF29" t="inlineStr"/>
-      <c r="AG29" t="inlineStr"/>
       <c r="AH29" t="n">
         <v>1</v>
       </c>
-      <c r="AI29" t="inlineStr"/>
-      <c r="AJ29" t="inlineStr"/>
-      <c r="AK29" t="inlineStr"/>
-      <c r="AL29" t="inlineStr"/>
-      <c r="AM29" t="inlineStr"/>
-      <c r="AN29" t="inlineStr"/>
-      <c r="AO29" t="inlineStr"/>
-      <c r="AP29" t="inlineStr"/>
       <c r="AQ29" t="n">
         <v>0</v>
       </c>
-      <c r="AR29" t="inlineStr"/>
-      <c r="AS29" t="inlineStr"/>
-      <c r="AT29" t="inlineStr"/>
-      <c r="AU29" t="inlineStr"/>
-      <c r="AV29" t="inlineStr"/>
-      <c r="AW29" t="inlineStr"/>
-      <c r="AX29" t="inlineStr"/>
-      <c r="AY29" t="inlineStr"/>
-      <c r="AZ29" t="inlineStr"/>
-      <c r="BA29" t="inlineStr"/>
-      <c r="BB29" t="inlineStr"/>
-      <c r="BC29" t="inlineStr"/>
-      <c r="BD29" t="inlineStr"/>
-      <c r="BE29" t="inlineStr"/>
-      <c r="BF29" t="inlineStr"/>
       <c r="BG29" t="n">
         <v>1</v>
       </c>
-      <c r="BH29" t="inlineStr"/>
-      <c r="BI29" t="inlineStr"/>
-      <c r="BJ29" t="inlineStr"/>
-      <c r="BK29" t="inlineStr"/>
-      <c r="BL29" t="inlineStr"/>
-      <c r="BM29" t="inlineStr"/>
-      <c r="BN29" t="inlineStr"/>
-      <c r="BO29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:15:06</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0525_local_hard</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="D30" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="F30" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" t="n">
+        <v>14</v>
+      </c>
+      <c r="U30" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-26 11:21:17</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0526_local_hard</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F31" t="n">
+        <v>4</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>4</v>
+      </c>
+      <c r="X31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-26 11:21:31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0526_local_hard</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>4</v>
+      </c>
+      <c r="X32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-26 11:21:39</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0526_local_hard_half</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="D33" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="F33" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" t="n">
+        <v>17</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-26 11:23:13</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0526_local_hard_half</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="D34" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="F34" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" t="n">
+        <v>17</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG34" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK34" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO34" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:11:15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0526_few_tc2</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="D35" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="F35" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="G35" t="n">
+        <v>6</v>
+      </c>
+      <c r="H35" t="n">
+        <v>9</v>
+      </c>
+      <c r="R35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK35" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-27 14:18:16</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0527_test</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>100</v>
+      </c>
+      <c r="D36" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>4</v>
+      </c>
+      <c r="G36" t="n">
+        <v>9</v>
+      </c>
+      <c r="H36" t="n">
+        <v>9</v>
+      </c>
+      <c r="R36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ36" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA36" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK36" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS36" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT36" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-28 01:01:27</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0527_local_hard</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>24.49</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F37" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="G37" t="n">
+        <v>12</v>
+      </c>
+      <c r="H37" t="n">
+        <v>49</v>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="n">
+        <v>1</v>
+      </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="n">
+        <v>0</v>
+      </c>
+      <c r="U37" t="n">
+        <v>0</v>
+      </c>
+      <c r="V37" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" t="inlineStr"/>
+      <c r="X37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="inlineStr"/>
+      <c r="AI37" t="inlineStr"/>
+      <c r="AJ37" t="inlineStr"/>
+      <c r="AK37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG37" t="inlineStr"/>
+      <c r="BH37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK37" t="inlineStr"/>
+      <c r="BL37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP37" t="inlineStr"/>
+      <c r="BQ37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS37" t="inlineStr"/>
+      <c r="BT37" t="inlineStr"/>
+      <c r="BU37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW37" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY37" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4943,7 +6133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:W20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.9"/>
   <sheetData>
     <row r="1">
@@ -6176,6 +7366,81 @@
         <v>1</v>
       </c>
       <c r="I19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-11 16:36:35</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0511_bank</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="D20" t="n">
+        <v>53.33</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" t="n">
+        <v>10</v>
+      </c>
+      <c r="H20" t="n">
+        <v>15</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" t="n">
+        <v>1</v>
+      </c>
+      <c r="P20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="n">
+        <v>1</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>1</v>
+      </c>
+      <c r="W20" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>